<commit_message>
[feat] 1.2 Beta R8
Features
Add Ceramic, Cobblestone, Mini Diamond Plate droopers
Add Changelog menu that is an button
Store menu is now created at runtime loaded once improving performance

Changes
Remove menu controller code from game.gd as it makes zero sense and use it as an class instead
Add enemies, coins earned stats
Add skip disclaimer option
Update Additional Music DLC Download link
Add Coins earned counter that resets each 10 seconds
Add sound when the changelog opens
Add changelog sprite
Open the changelog menu when savefile is new
Add 1.2 article in changelog menu and update it (english)
Add go back to the top button in changelog menu

Fixes
Fix Music DLC Crashing game

KNOWN BUGS
The previous item buy button will still be seen after switching page
</commit_message>
<xml_diff>
--- a/data/languages/languages.xlsx
+++ b/data/languages/languages.xlsx
@@ -67,7 +67,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="195">
   <si>
     <t xml:space="preserve">key</t>
   </si>
@@ -316,6 +316,96 @@
   </si>
   <si>
     <t xml:space="preserve">Язик</t>
+  </si>
+  <si>
+    <t xml:space="preserve">skip_disclaimer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skip Disclaimer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Пропустить дисклеймер</t>
+  </si>
+  <si>
+    <t xml:space="preserve">skip_disclaimer_description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">If turned on Skips the disclaimer screen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Если включено то екран дисклеймера будет пропущен</t>
+  </si>
+  <si>
+    <t xml:space="preserve">changelog</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Сhangelog</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Изменения</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stats</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stats</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Статистика</t>
+  </si>
+  <si>
+    <t xml:space="preserve">enemies_killed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enemies killed: </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Врагов убито: </t>
+  </si>
+  <si>
+    <t xml:space="preserve">droopers_bought</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Droopers bought: </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Дроперов куплено:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">upgrades_bought</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Upgrades bought: </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Улучшенний куплено: </t>
+  </si>
+  <si>
+    <t xml:space="preserve">enemies_bought</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enemies bought: </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Врагов куплено: </t>
+  </si>
+  <si>
+    <t xml:space="preserve">coins_earned</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coins earned: </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Монет накоплено: </t>
+  </si>
+  <si>
+    <t xml:space="preserve">time_played</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Time played: </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Наиграно:</t>
   </si>
   <si>
     <t xml:space="preserve">credits</t>
@@ -703,7 +793,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -721,10 +811,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -851,7 +937,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C55"/>
+  <dimension ref="A1:C67"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="29.53"/>
@@ -1123,7 +1209,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="57.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="58" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
         <v>72</v>
       </c>
@@ -1167,14 +1253,14 @@
         <v>83</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="287.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="0" t="s">
+    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="B29" s="5" t="s">
+      <c r="B29" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="C29" s="5" t="s">
+      <c r="C29" s="1" t="s">
         <v>86</v>
       </c>
     </row>
@@ -1190,79 +1276,79 @@
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="1" t="s">
+      <c r="A31" s="0" t="s">
         <v>90</v>
       </c>
-      <c r="B31" s="1" t="s">
+      <c r="B31" s="0" t="s">
         <v>91</v>
       </c>
-      <c r="C31" s="1" t="s">
+      <c r="C31" s="0" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="1" t="s">
+      <c r="A32" s="0" t="s">
         <v>93</v>
       </c>
-      <c r="B32" s="1" t="s">
+      <c r="B32" s="0" t="s">
         <v>94</v>
       </c>
-      <c r="C32" s="3" t="s">
+      <c r="C32" s="0" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="1" t="s">
+      <c r="A33" s="0" t="s">
         <v>96</v>
       </c>
-      <c r="B33" s="1" t="s">
+      <c r="B33" s="0" t="s">
         <v>97</v>
       </c>
-      <c r="C33" s="1" t="s">
+      <c r="C33" s="0" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="1" t="s">
+      <c r="A34" s="0" t="s">
         <v>99</v>
       </c>
-      <c r="B34" s="1" t="s">
+      <c r="B34" s="0" t="s">
         <v>100</v>
       </c>
-      <c r="C34" s="1" t="s">
+      <c r="C34" s="0" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="1" t="s">
+      <c r="A35" s="0" t="s">
         <v>102</v>
       </c>
-      <c r="B35" s="1" t="s">
+      <c r="B35" s="0" t="s">
         <v>103</v>
       </c>
-      <c r="C35" s="1" t="s">
+      <c r="C35" s="0" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="1" t="s">
+      <c r="A36" s="0" t="s">
         <v>105</v>
       </c>
-      <c r="B36" s="1" t="s">
+      <c r="B36" s="0" t="s">
         <v>106</v>
       </c>
-      <c r="C36" s="1" t="s">
+      <c r="C36" s="0" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="1" t="s">
+      <c r="A37" s="0" t="s">
         <v>108</v>
       </c>
-      <c r="B37" s="1" t="s">
+      <c r="B37" s="0" t="s">
         <v>109</v>
       </c>
-      <c r="C37" s="1" t="s">
+      <c r="C37" s="0" t="s">
         <v>110</v>
       </c>
     </row>
@@ -1277,14 +1363,14 @@
         <v>113</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="398" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="B39" s="1" t="s">
+      <c r="B39" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="C39" s="1" t="s">
+      <c r="C39" s="3" t="s">
         <v>116</v>
       </c>
     </row>
@@ -1317,7 +1403,7 @@
       <c r="B42" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="C42" s="1" t="s">
+      <c r="C42" s="3" t="s">
         <v>125</v>
       </c>
     </row>
@@ -1398,14 +1484,14 @@
         <v>146</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="102.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="B50" s="3" t="s">
+      <c r="B50" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="C50" s="4" t="s">
+      <c r="C50" s="1" t="s">
         <v>149</v>
       </c>
     </row>
@@ -1463,6 +1549,126 @@
       <c r="C55" s="1" t="s">
         <v>164</v>
       </c>
+    </row>
+    <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="C58" s="1" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="103.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="B60" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="C60" s="4" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="C61" s="1" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="C63" s="1" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="C64" s="1" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="C65" s="1" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="0"/>
+      <c r="B66" s="0"/>
+      <c r="C66" s="0"/>
+    </row>
+    <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="0"/>
+      <c r="B67" s="0"/>
+      <c r="C67" s="0"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>